<commit_message>
D04: author's gap analysis (final), draft note removed; AI-use statement updated
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01CsLFgwnuQK8yyd4UPD8vPc
</commit_message>
<xml_diff>
--- a/04_Systematic_Review/synthesis/D04_extraction_and_gaps.xlsx
+++ b/04_Systematic_Review/synthesis/D04_extraction_and_gaps.xlsx
@@ -2,16 +2,15 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
-  <workbookProtection/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" tabRatio="600" firstSheet="0" activeTab="1" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Extraction_matrix" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gap_analysis" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <calcPr calcId="0" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
@@ -29,7 +28,7 @@
     <font>
       <name val="Arial"/>
       <b val="1"/>
-      <color rgb="00FFFFFF"/>
+      <color rgb="FFFFFFFF"/>
       <sz val="9"/>
     </font>
     <font>
@@ -39,7 +38,7 @@
     <font>
       <name val="Arial"/>
       <i val="1"/>
-      <color rgb="00C00000"/>
+      <color rgb="FFC00000"/>
       <sz val="9"/>
     </font>
   </fonts>
@@ -52,7 +51,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="001F3864"/>
+        <fgColor rgb="FF1F3864"/>
       </patternFill>
     </fill>
   </fills>
@@ -66,17 +65,18 @@
     </border>
     <border>
       <left style="thin">
-        <color rgb="00BFBFBF"/>
+        <color rgb="FFBFBFBF"/>
       </left>
       <right style="thin">
-        <color rgb="00BFBFBF"/>
+        <color rgb="FFBFBFBF"/>
       </right>
       <top style="thin">
-        <color rgb="00BFBFBF"/>
+        <color rgb="FFBFBFBF"/>
       </top>
       <bottom style="thin">
-        <color rgb="00BFBFBF"/>
+        <color rgb="FFBFBFBF"/>
       </bottom>
+      <diagonal/>
     </border>
   </borders>
   <cellStyleXfs count="1">
@@ -93,7 +93,7 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
@@ -457,23 +457,21 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:L11"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
     <col width="7" customWidth="1" min="2" max="2"/>
     <col width="20" customWidth="1" min="3" max="3"/>
     <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="22" customWidth="1" min="5" max="5"/>
-    <col width="22" customWidth="1" min="6" max="6"/>
+    <col width="22" customWidth="1" min="5" max="6"/>
     <col width="26" customWidth="1" min="7" max="7"/>
     <col width="16" customWidth="1" min="8" max="8"/>
     <col width="30" customWidth="1" min="9" max="9"/>
     <col width="28" customWidth="1" min="10" max="10"/>
-    <col width="30" customWidth="1" min="11" max="11"/>
-    <col width="30" customWidth="1" min="12" max="12"/>
+    <col width="30" customWidth="1" min="11" max="12"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" ht="36" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
           <t>ID</t>
@@ -535,7 +533,7 @@
         </is>
       </c>
     </row>
-    <row r="2">
+    <row r="2" ht="36" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
           <t>S1</t>
@@ -597,7 +595,7 @@
         </is>
       </c>
     </row>
-    <row r="3">
+    <row r="3" ht="24" customHeight="1">
       <c r="A3" s="2" t="inlineStr">
         <is>
           <t>S2</t>
@@ -659,7 +657,7 @@
         </is>
       </c>
     </row>
-    <row r="4">
+    <row r="4" ht="36" customHeight="1">
       <c r="A4" s="2" t="inlineStr">
         <is>
           <t>S3</t>
@@ -721,7 +719,7 @@
         </is>
       </c>
     </row>
-    <row r="5">
+    <row r="5" ht="36" customHeight="1">
       <c r="A5" s="2" t="inlineStr">
         <is>
           <t>S4</t>
@@ -783,7 +781,7 @@
         </is>
       </c>
     </row>
-    <row r="6">
+    <row r="6" ht="24" customHeight="1">
       <c r="A6" s="2" t="inlineStr">
         <is>
           <t>S5</t>
@@ -845,7 +843,7 @@
         </is>
       </c>
     </row>
-    <row r="7">
+    <row r="7" ht="36" customHeight="1">
       <c r="A7" s="2" t="inlineStr">
         <is>
           <t>S6</t>
@@ -907,7 +905,7 @@
         </is>
       </c>
     </row>
-    <row r="8">
+    <row r="8" ht="36" customHeight="1">
       <c r="A8" s="2" t="inlineStr">
         <is>
           <t>S7</t>
@@ -969,7 +967,7 @@
         </is>
       </c>
     </row>
-    <row r="9">
+    <row r="9" ht="36" customHeight="1">
       <c r="A9" s="2" t="inlineStr">
         <is>
           <t>S8</t>
@@ -1031,7 +1029,7 @@
         </is>
       </c>
     </row>
-    <row r="10">
+    <row r="10" ht="36" customHeight="1">
       <c r="A10" s="2" t="inlineStr">
         <is>
           <t>S9</t>
@@ -1093,7 +1091,7 @@
         </is>
       </c>
     </row>
-    <row r="11">
+    <row r="11" ht="36" customHeight="1">
       <c r="A11" s="2" t="inlineStr">
         <is>
           <t>S10</t>
@@ -1167,7 +1165,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:E7"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
     <col width="70" customWidth="1" min="2" max="2"/>
@@ -1176,7 +1174,7 @@
     <col width="22" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" ht="24" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Gap type (Session 4)</t>
@@ -1203,7 +1201,7 @@
         </is>
       </c>
     </row>
-    <row r="2">
+    <row r="2" ht="72" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
           <t>Knowledge</t>
@@ -1211,26 +1209,26 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>No study targets the student's decision of WHETHER to delegate academic work to the LLM; all ten scaffold reasoning within a learning task (writing, reflection, SRL, problem solving). Delegation-related outcomes appear only as AI dependency (S5) and reduced direct uptake / AI literacy (S7).</t>
+          <t>None of the 10 included studies trains or scaffolds the student's decision of whether to delegate a task to AI; all 10 scaffold reasoning or reflection within an already-assigned task (post-assignment reflection in S1; non-directive process prompts, hints, or withholding direct answers in S2, S3, S7, S8, S10; eliciting or metacognitive/co-regulation questions in S4, S5, S9; target-setting and task decomposition in S6). The closest are S5 (measures GenAI dependency) and S7 (AI literacy), but neither scaffolds the decision itself.</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>S5 Yuan (2026); S7 Aldamen et al. (2026); S3 Lee et al. (2024)</t>
+          <t>0/10 train the delegation decision (10/10 scaffold within-task reasoning) — S1, S2, S3, S4, S5, S6, S7, S8, S9, S10</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>RQ1/RQ2: scaffolding the delegation decision itself</t>
+          <t>My agent and protocol will explicitly scaffold and evaluate the student's prior decision of whether and what to delegate to the LLM before task execution.</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>High (absence observed in the 10 included; limited by the cap)</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
+          <t>Medium — the search strategy did not include delegation-specific terms and the 10-study prioritisation cap left full texts unassessed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="96" customHeight="1">
       <c r="A3" s="2" t="inlineStr">
         <is>
           <t>Methodological</t>
@@ -1238,26 +1236,26 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Evidence that effects persist without the tool is scarce: only S7 tests delayed transfer without AI and S5 tests writing without GenAI; most outcomes are self-reported and immediate. Tool configuration is often not reported (S2, S6 do not name the LLM; S9 prompts only in supplement), limiting replication.</t>
+          <t>Only 5 of 10 included studies compare the scaffolded tool against a plain LLM (C1: S3, S4, S6, S7, S9). The 4 C2-only studies (S1, S2, S8, S10) compare against no AI or teacher feedback, confounding AI access with scaffolding, and the C3 study (S5) compares two scaffolds; neither design can isolate the scaffolding effect. Only 2 of 10 report a delayed measure (S3, delayed knowledge test; S7, delayed transfer without AI).</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>S7; S5; S2 Hou et al. (2026); S6 Niez et al. (2026); S9 Yang et al. (2025)</t>
+          <t>5/10 include C1 (S3, S4, S6, S7, S9); 4/10 C2 only (S1, S2, S8, S10); 1/10 C3 (S5); S7 has both C1 and C2 arms. 2/10 report a delayed measure (S3, S7).</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>Measure unassisted performance and dependence after the intervention; publish prompts</t>
+          <t>My evaluation will include an unrestricted plain-LLM condition (C1) to isolate the scaffolding effect, and an unassisted post-test.</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>High</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
+          <t>High for comparator type (dedicated extraction column for all 10); Medium for measurement timing (no timing column; delayed measures recorded only where reported). Bounded by the 10-study cap.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="96" customHeight="1">
       <c r="A4" s="2" t="inlineStr">
         <is>
           <t>Contextual</t>
@@ -1265,26 +1263,26 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Studies come mainly from East Asia (S2, S3, S5, S9) and EFL/CS courses; the only Spanish-language study (S8) is in mathematics and its setting is inconsistently reported. No study involves Peruvian students.</t>
+          <t>None of the 10 included studies involves students in Peru, and only 1 is set in Latin America (S8), which is also the only Spanish-language study; the evidence is concentrated in Asia (6/10) and in language and computing courses (7/10).</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>S8 Macías Hinojoza et al. (2026); S9; S5</t>
+          <t>0/10 Peru; 1/10 Latin America (S8, Ecuador; text also mentions Spain); 6/10 Asia (China: S2, S5, S9; Taiwan: S3; Philippines: S6; Jordan: S7); Canada: S1; Europe, country not stated: S4; country not stated: S10. Disciplines: EFL/ESL/English 4/10 (S5, S6, S7, S9); CS/Python 3/10 (S1, S2, S4); engineering 2/10 (S8, S10); chemistry 1/10 (S3).</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>Peruvian undergraduates; Spanish-language tool</t>
+          <t>My evaluation will test a Spanish-language agent with undergraduates at a Peruvian university.</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Medium (country not reported for S10; cap may hide studies)</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
+          <t>Medium — country is not stated in the extracted text for S10 (and S4 states only Europe; S8 has site inconsistency), and the 10-study cap may exclude regional studies.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="96" customHeight="1">
       <c r="A5" s="2" t="inlineStr">
         <is>
           <t>Theoretical</t>
@@ -1292,31 +1290,28 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>Designs rest on self-regulated or co-regulated learning and metacognition (S1, S5, S9) but no framework explains why tool-level scaffolding improves process measures without consistent gains in performance (S1 exam n.s.; S5 writing n.s.). No included study draws on ethics (e.g., virtue ethics/phronesis) as a design basis.</t>
+          <t>All 10 included studies frame their outcomes in cognitive, metacognitive, motivational or self-regulation terms, or in task performance alone; none of the 10 measures academic integrity or any ethical outcome, although academic integrity was a pre-specified outcome of interest (I4), and none grounds its scaffolding in practical judgment (phronesis) about when and what to delegate to AI. Transfer to unassisted performance is mixed: self-reported or process gains are not matched by unassisted performance in S1 and S5.</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>S1 Kumar et al. (2024); S5; S9</t>
+          <t>7/10 measure cognitive, metacognitive, motivational or SRL constructs (S1 self-confidence; S2 MAI; S3 SRL, HOTS; S4 reflection, JoL accuracy; S5 SRL, GenAI dependency; S6 SRL, engagement; S7 AI literacy); 3/10 measure task performance only (S8, S9, S10; S9 frames its scaffold as co-regulation). 0/10 measure academic integrity or an ethical outcome. 7/10 report objective performance gains (S2, S3, S6, S7, S8, S9, S10); 2/10 do not (S1 exam n.s.; S5 writing without AI n.s.); S4 has no performance test.</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>Virtue-ethics design theory for scaffolding judgment</t>
+          <t>My protocol and agent will draw on virtue ethics (practical judgment / phronesis) to link metacognitive scaffolding with the student's autonomous judgment about when to turn to AI, and will measure product integrity and performance without the tool.</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>Medium</t>
-        </is>
-      </c>
-    </row>
+          <t>Low to Medium: the matrix has no theoretical-framework column (constructs are inferred from the Outcomes and Scaffolding columns), the search string had no ethics terms, and the 10-study cap left full texts unassessed. The absence of integrity outcomes is the firmer claim, since 'academic integrity' was a search term.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6"/>
     <row r="7">
-      <c r="A7" s="3" t="inlineStr">
-        <is>
-          <t>DRAFT for the author: statements must be checked and rewritten by the author before submission. Gaps are bounded by a 10-study rapid review with a prioritisation cap.</t>
-        </is>
-      </c>
+      <c r="A7" s="3" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>